<commit_message>
Ajuste código de alteração pedido de frete - campo CC
</commit_message>
<xml_diff>
--- a/Planilhas/Pedidos - Copia.xlsx
+++ b/Planilhas/Pedidos - Copia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\junio\OneDrive\Área de Trabalho\Documentos\Scripts Github\automations\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E139DFC-C5C3-44A7-B613-3425CED342B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE548F8C-954E-4193-9A59-AF3DE585B7C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B22F4247-8A78-4CA2-917D-234C68224E18}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="4">
   <si>
     <t>Item</t>
   </si>
@@ -84,7 +84,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="3">
     <dxf>
       <font>
         <b val="0"/>
@@ -132,20 +132,6 @@
       </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -160,8 +146,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C4F11308-4C43-48B9-BA07-AEB362118F73}" name="Tabela1" displayName="Tabela1" ref="A1:C2" totalsRowShown="0" dataDxfId="3">
-  <autoFilter ref="A1:C2" xr:uid="{C4F11308-4C43-48B9-BA07-AEB362118F73}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C4F11308-4C43-48B9-BA07-AEB362118F73}" name="Tabela1" displayName="Tabela1" ref="A1:C37" totalsRowShown="0">
+  <autoFilter ref="A1:C37" xr:uid="{C4F11308-4C43-48B9-BA07-AEB362118F73}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D0BC8C79-FDF1-4144-B598-1BCD4BB7CFD1}" name="Pedidos" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{3D9316E3-CFBE-4A9E-8B75-E0BF8E30E135}" name="Item" dataDxfId="1"/>
@@ -468,7 +454,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C176DAE8-01D4-4562-9DC5-3FF54C0846F5}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
@@ -488,12 +474,397 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>4500030627</v>
+        <v>4500031354</v>
       </c>
       <c r="B2">
         <v>10</v>
       </c>
       <c r="C2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>4500031355</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>4500031356</v>
+      </c>
+      <c r="B4">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4500031357</v>
+      </c>
+      <c r="B5">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>4500031358</v>
+      </c>
+      <c r="B6">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>4500031368</v>
+      </c>
+      <c r="B7">
+        <v>10</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>4500031369</v>
+      </c>
+      <c r="B8">
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>4500031377</v>
+      </c>
+      <c r="B9">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>4500031378</v>
+      </c>
+      <c r="B10">
+        <v>10</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>4500031379</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>4500031380</v>
+      </c>
+      <c r="B12">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>4500031383</v>
+      </c>
+      <c r="B13">
+        <v>10</v>
+      </c>
+      <c r="C13" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>4500031385</v>
+      </c>
+      <c r="B14">
+        <v>10</v>
+      </c>
+      <c r="C14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>4500031386</v>
+      </c>
+      <c r="B15">
+        <v>10</v>
+      </c>
+      <c r="C15" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>4500031387</v>
+      </c>
+      <c r="B16">
+        <v>10</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>4500031388</v>
+      </c>
+      <c r="B17">
+        <v>10</v>
+      </c>
+      <c r="C17" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>4500031389</v>
+      </c>
+      <c r="B18">
+        <v>10</v>
+      </c>
+      <c r="C18" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>4500031390</v>
+      </c>
+      <c r="B19">
+        <v>10</v>
+      </c>
+      <c r="C19" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>4500031422</v>
+      </c>
+      <c r="B20">
+        <v>10</v>
+      </c>
+      <c r="C20" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>4500031423</v>
+      </c>
+      <c r="B21">
+        <v>10</v>
+      </c>
+      <c r="C21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>4500031424</v>
+      </c>
+      <c r="B22">
+        <v>10</v>
+      </c>
+      <c r="C22" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>4500031425</v>
+      </c>
+      <c r="B23">
+        <v>10</v>
+      </c>
+      <c r="C23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>4500031426</v>
+      </c>
+      <c r="B24">
+        <v>10</v>
+      </c>
+      <c r="C24" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>4500031427</v>
+      </c>
+      <c r="B25">
+        <v>10</v>
+      </c>
+      <c r="C25" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>4500031428</v>
+      </c>
+      <c r="B26">
+        <v>10</v>
+      </c>
+      <c r="C26" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>4500031429</v>
+      </c>
+      <c r="B27">
+        <v>10</v>
+      </c>
+      <c r="C27" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>4500031430</v>
+      </c>
+      <c r="B28">
+        <v>10</v>
+      </c>
+      <c r="C28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>4500031431</v>
+      </c>
+      <c r="B29">
+        <v>10</v>
+      </c>
+      <c r="C29" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>4500031432</v>
+      </c>
+      <c r="B30">
+        <v>10</v>
+      </c>
+      <c r="C30" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>4500031433</v>
+      </c>
+      <c r="B31">
+        <v>10</v>
+      </c>
+      <c r="C31" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>4500031434</v>
+      </c>
+      <c r="B32">
+        <v>10</v>
+      </c>
+      <c r="C32" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>4500031435</v>
+      </c>
+      <c r="B33">
+        <v>10</v>
+      </c>
+      <c r="C33" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>4500031436</v>
+      </c>
+      <c r="B34">
+        <v>10</v>
+      </c>
+      <c r="C34" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>4500031437</v>
+      </c>
+      <c r="B35">
+        <v>10</v>
+      </c>
+      <c r="C35" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>4500031438</v>
+      </c>
+      <c r="B36">
+        <v>10</v>
+      </c>
+      <c r="C36" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>4500031439</v>
+      </c>
+      <c r="B37">
+        <v>10</v>
+      </c>
+      <c r="C37" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>